<commit_message>
Refresh parity workbook metadata after review gates
The workbook status counts remain unchanged, but the repo evidence baseline advanced through Slice 6 guard migrations and review-gate packets. This refreshes workbook metadata to record the post-review baseline through commit 1ac2da7 and migration sequence 537 without promoting any GAP or PARTIAL rows.

Constraint: Workbook statuses must remain unchanged because provider/manual/finance closure evidence is still missing.

Rejected: Updating open rows to BUILT from readiness gates | decision packets explicitly prohibit that promotion.

Confidence: high

Scope-risk: narrow

Directive: Treat this as a metadata/evidence refresh only, not row closure.

Tested: node .omx/tmp/parity-review/verify_workbook.mjs

Tested: shasum -a 256 desktop and repo workbook copies matched

Tested: git diff --check

Not-tested: Opening workbook manually in Excel after metadata refresh
</commit_message>
<xml_diff>
--- a/docs/IntelliDealer/_Manifests/QEP_Parity_Worksheet.xlsx
+++ b/docs/IntelliDealer/_Manifests/QEP_Parity_Worksheet.xlsx
@@ -739,7 +739,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Reviewed: 2026-05-04   |   Repo HEAD: a4bd0e7   |   Statuses updated from current QEP repo evidence</t>
+          <t>Reviewed: 2026-05-04   |   Repo HEAD: 1ac2da7   |   Statuses unchanged; post-review gate evidence updated through migration 537</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="33">
@@ -2927,13 +2927,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>QEP Parity Worksheet Status Review</t>
         </is>
       </c>
-      <c r="B1" s="25" t="n"/>
-      <c r="C1" s="25" t="n"/>
+      <c r="B1" s="28" t="n"/>
+      <c r="C1" s="28" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="27" t="inlineStr">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="B3" s="27" t="inlineStr">
         <is>
-          <t>a4bd0e7</t>
+          <t>1ac2da7</t>
         </is>
       </c>
       <c r="C3" s="27" t="n"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Prospect Board JD Quote II/JD PO workflows; equipment sale reversal by stock number.</t>
+          <t>Prospect Board JD Quote II/JD PO workflows; equipment sale reversal by stock number (foundation/readiness guard present; reversal execution policy-gated).</t>
         </is>
       </c>
       <c r="C14" s="27" t="n"/>
@@ -3134,7 +3134,11 @@
       </c>
       <c r="C16" s="27" t="n"/>
     </row>
-    <row r="17"/>
+    <row r="17">
+      <c r="A17" s="27" t="n"/>
+      <c r="B17" s="27" t="n"/>
+      <c r="C17" s="27" t="n"/>
+    </row>
     <row r="18">
       <c r="A18" s="42" t="inlineStr">
         <is>
@@ -3301,7 +3305,7 @@
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>Verify migrations, provider readiness, segment gates, workbook formula scan/rendering, and desktop/repo SHA sync.</t>
+          <t>Verify migrations, provider readiness, segment gates, workbook formula scan/rendering, desktop/repo SHA sync, and that decision packets have closure evidence.</t>
         </is>
       </c>
     </row>

</xml_diff>